<commit_message>
Include User Allowed Locations Access
</commit_message>
<xml_diff>
--- a/uploads/UPLOAD-TEMPLATE/STAFFS-UPLOAD-TEMPLATE.xlsx
+++ b/uploads/UPLOAD-TEMPLATE/STAFFS-UPLOAD-TEMPLATE.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\OSH-Backend\uploads\UPLOAD-TEMPLATE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCA6B5C2-C576-40B6-A7E2-D543FB146080}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D38B74D3-0BAA-4DFB-A369-6B8B6F8C2A63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{8DE630E0-0B89-4DDE-A92E-DF514EA9A919}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
   <si>
     <t>Middle Name</t>
   </si>
@@ -115,12 +115,6 @@
   </si>
   <si>
     <t>Category Type</t>
-  </si>
-  <si>
-    <t>Allowance</t>
-  </si>
-  <si>
-    <t>Salary Rate</t>
   </si>
   <si>
     <t>INVENTORY AUDIT</t>
@@ -543,7 +537,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FAE589B1-C7BA-44D4-9E29-919A5892AA9B}">
-  <dimension ref="A1:AC4"/>
+  <dimension ref="A1:AA4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="55.85546875" bestFit="1" customWidth="1"/>
@@ -555,24 +549,24 @@
     <col min="8" max="8" width="30.7109375" customWidth="1"/>
     <col min="9" max="9" width="25" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="29.28515625" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="29.28515625" customWidth="1"/>
-    <col min="15" max="15" width="49.85546875" customWidth="1"/>
-    <col min="16" max="16" width="29.7109375" customWidth="1"/>
-    <col min="17" max="18" width="39.42578125" customWidth="1"/>
-    <col min="19" max="19" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="14.85546875" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="20.140625" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="23" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="22.28515625" customWidth="1"/>
-    <col min="28" max="28" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="17.28515625" customWidth="1"/>
+    <col min="11" max="12" width="29.28515625" customWidth="1"/>
+    <col min="13" max="13" width="49.85546875" customWidth="1"/>
+    <col min="14" max="14" width="29.7109375" customWidth="1"/>
+    <col min="15" max="16" width="39.42578125" customWidth="1"/>
+    <col min="17" max="17" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="23" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="22.28515625" customWidth="1"/>
+    <col min="26" max="26" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="17.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>27</v>
       </c>
@@ -586,7 +580,7 @@
         <v>0</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="F1" s="2" t="s">
         <v>4</v>
@@ -607,69 +601,63 @@
         <v>29</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="M1" s="2" t="s">
-        <v>31</v>
+        <v>9</v>
       </c>
       <c r="N1" s="2" t="s">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="O1" s="2" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="P1" s="2" t="s">
-        <v>10</v>
+        <v>36</v>
       </c>
       <c r="Q1" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="R1" s="2" t="s">
-        <v>38</v>
+        <v>13</v>
       </c>
       <c r="S1" s="2" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="T1" s="2" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="U1" s="2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="V1" s="2" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="W1" s="2" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="X1" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="Y1" s="2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="Z1" s="2" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="AA1" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="AB1" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="AC1" s="2" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
-    <row r="2" spans="1:29" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B2" t="s">
         <v>24</v>
       </c>
       <c r="C2" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F2">
         <v>55555</v>
@@ -687,31 +675,31 @@
         <v>22</v>
       </c>
       <c r="K2" t="s">
+        <v>30</v>
+      </c>
+      <c r="L2" t="s">
+        <v>31</v>
+      </c>
+      <c r="M2" t="s">
         <v>32</v>
       </c>
-      <c r="L2">
-        <v>5312</v>
-      </c>
-      <c r="M2">
-        <v>5221</v>
-      </c>
-      <c r="N2" t="s">
-        <v>33</v>
-      </c>
-      <c r="O2" t="s">
-        <v>34</v>
-      </c>
-      <c r="P2">
+      <c r="N2">
         <v>1234567890</v>
       </c>
+      <c r="O2" s="5">
+        <v>123456789</v>
+      </c>
+      <c r="P2" s="5">
+        <v>123456789012</v>
+      </c>
       <c r="Q2" s="5">
-        <v>123456789</v>
-      </c>
-      <c r="R2" s="5">
         <v>123456789012</v>
       </c>
-      <c r="S2" s="5">
-        <v>123456789012</v>
+      <c r="S2" s="3">
+        <v>46170</v>
+      </c>
+      <c r="T2" s="3">
+        <v>46170</v>
       </c>
       <c r="U2" s="3">
         <v>46170</v>
@@ -728,22 +716,16 @@
       <c r="Y2" s="3">
         <v>46170</v>
       </c>
-      <c r="Z2" s="3">
-        <v>46170</v>
-      </c>
-      <c r="AA2" s="3">
-        <v>46170</v>
-      </c>
-      <c r="AC2" t="b">
+      <c r="AA2" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="4" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>3</v>
       </c>

</xml_diff>